<commit_message>
Actualizar documentos y trasladar entregables a Fase 2
</commit_message>
<xml_diff>
--- a/Evaluación-fase-1/Bomberos KPI Y KRI.xlsx
+++ b/Evaluación-fase-1/Bomberos KPI Y KRI.xlsx
@@ -11,6 +11,36 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment authorId="0" ref="C1">
+      <text>
+        <t xml:space="preserve">Antes de clasificar resultados porcentuales, acordar el número de decimales, el redondeo y los extremos de cada banda. Conservar las metas y bandas existentes hasta que el equipo valide ese criterio.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment authorId="0" ref="C1">
+      <text>
+        <t xml:space="preserve">Identificar fecha de corte, universo y fórmula de medición. Acordar decimales y extremos de las bandas porcentuales sin modificar los umbrales existentes por esta revisión documental.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="246">
   <si>
@@ -20,18 +50,18 @@
     <t>KRI</t>
   </si>
   <si>
+    <t>Unidad</t>
+  </si>
+  <si>
+    <t>Meta</t>
+  </si>
+  <si>
+    <t>Preventivo</t>
+  </si>
+  <si>
     <t>KPI</t>
   </si>
   <si>
-    <t>Unidad</t>
-  </si>
-  <si>
-    <t>Meta</t>
-  </si>
-  <si>
-    <t>Preventivo</t>
-  </si>
-  <si>
     <t>Critico</t>
   </si>
   <si>
@@ -53,45 +83,45 @@
     <t>KRI-01</t>
   </si>
   <si>
+    <t>Requisitos pendientes de aclaracion</t>
+  </si>
+  <si>
+    <t>Cantidad</t>
+  </si>
+  <si>
     <t>KPI-01</t>
   </si>
   <si>
-    <t>Requisitos pendientes de aclaracion</t>
+    <t>0</t>
   </si>
   <si>
     <t>Cumplimiento cronograma</t>
   </si>
   <si>
-    <t>Cantidad</t>
+    <t>1-2</t>
+  </si>
+  <si>
+    <t>≥3</t>
   </si>
   <si>
     <t>%</t>
   </si>
   <si>
-    <t>0</t>
+    <t>Semanal</t>
   </si>
   <si>
     <t>≥90%</t>
   </si>
   <si>
-    <t>1-2</t>
+    <t>Mauricio</t>
   </si>
   <si>
     <t>80%-89%</t>
   </si>
   <si>
-    <t>≥3</t>
-  </si>
-  <si>
     <t>&lt;80%</t>
   </si>
   <si>
-    <t>Semanal</t>
-  </si>
-  <si>
-    <t>Mauricio</t>
-  </si>
-  <si>
     <t>Define como se mide el indicador KPI o KRI</t>
   </si>
   <si>
@@ -101,48 +131,63 @@
     <t>KRI-02</t>
   </si>
   <si>
+    <t>Cambios de alcance sin evaluar</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>≥2</t>
+  </si>
+  <si>
     <t>KPI-02</t>
   </si>
   <si>
-    <t>Cambios de alcance sin evaluar</t>
-  </si>
-  <si>
     <t>Cumplimiento EDT y entregables</t>
   </si>
   <si>
+    <t>Valor objetivo esperado para considerar el indicador dentro del nivel aceptable</t>
+  </si>
+  <si>
+    <t>Historias Done ≥90% y defectos criticos 0</t>
+  </si>
+  <si>
     <t>≥95%</t>
   </si>
   <si>
-    <t>1</t>
+    <t>KRI-03</t>
   </si>
   <si>
     <t>85%-94%</t>
   </si>
   <si>
-    <t>≥2</t>
+    <t>Reglas operativas sin validar</t>
   </si>
   <si>
     <t>&lt;85%</t>
   </si>
   <si>
-    <t>Valor objetivo esperado para considerar el indicador dentro del nivel aceptable</t>
-  </si>
-  <si>
-    <t>Historias Done ≥90% y defectos criticos 0</t>
-  </si>
-  <si>
-    <t>KRI-03</t>
+    <t>Nivel Preventivo</t>
+  </si>
+  <si>
+    <t>Rango de advertencia que requiere seguimiento antes de llegar al nivel critico</t>
+  </si>
+  <si>
+    <t>Bloqueos activos 1 y pruebas no ejecutadas entre 11% y 20%</t>
   </si>
   <si>
     <t>KPI-03</t>
   </si>
   <si>
-    <t>Reglas operativas sin validar</t>
-  </si>
-  <si>
     <t>Cumplimiento Sprint Goal</t>
   </si>
   <si>
+    <t>KRI-04</t>
+  </si>
+  <si>
+    <t>Historias sin criterios verificables</t>
+  </si>
+  <si>
     <t>100%</t>
   </si>
   <si>
@@ -152,163 +197,184 @@
     <t>Por Sprint</t>
   </si>
   <si>
-    <t>Nivel Preventivo</t>
-  </si>
-  <si>
-    <t>Rango de advertencia que requiere seguimiento antes de llegar al nivel critico</t>
-  </si>
-  <si>
-    <t>Bloqueos activos 1 y pruebas no ejecutadas entre 11% y 20%</t>
-  </si>
-  <si>
-    <t>KRI-04</t>
+    <t>Nivel Critico</t>
+  </si>
+  <si>
+    <t>Nivel que requiere accion correctiva porque compromete plazo calidad seguridad y operacion</t>
+  </si>
+  <si>
+    <t>Defectos criticos ≥2 y trabajo pendiente &gt;20%</t>
+  </si>
+  <si>
+    <t>KRI-05</t>
+  </si>
+  <si>
+    <t>Fallas de integracion frontend y backend</t>
   </si>
   <si>
     <t>KPI-04</t>
   </si>
   <si>
-    <t>Historias sin criterios verificables</t>
-  </si>
-  <si>
     <t>Historias Done</t>
   </si>
   <si>
+    <t>Alexander</t>
+  </si>
+  <si>
+    <t>Indica cada cuanto se revisa el indicador</t>
+  </si>
+  <si>
+    <t>Diario semanal por Sprint release y final</t>
+  </si>
+  <si>
     <t>75%-89%</t>
   </si>
   <si>
     <t>&lt;75%</t>
   </si>
   <si>
+    <t>KRI-06</t>
+  </si>
+  <si>
+    <t>Cambios tardios del modelo de datos</t>
+  </si>
+  <si>
     <t>Equipo</t>
   </si>
   <si>
-    <t>Nivel Critico</t>
-  </si>
-  <si>
-    <t>Nivel que requiere accion correctiva porque compromete plazo calidad seguridad y operacion</t>
-  </si>
-  <si>
-    <t>Defectos criticos ≥2 y trabajo pendiente &gt;20%</t>
-  </si>
-  <si>
-    <t>KRI-05</t>
-  </si>
-  <si>
     <t>KPI-05</t>
   </si>
   <si>
-    <t>Fallas de integracion frontend y backend</t>
-  </si>
-  <si>
     <t>Cumplimiento Definition of Done</t>
   </si>
   <si>
+    <t>Paulo</t>
+  </si>
+  <si>
     <t>90%-99%</t>
   </si>
   <si>
+    <t>Persona o equipo encargado de revisar el indicador y coordinar acciones</t>
+  </si>
+  <si>
+    <t>Mauricio Paulo Alexander y Equipo</t>
+  </si>
+  <si>
     <t>&lt;90%</t>
   </si>
   <si>
-    <t>Alexander</t>
-  </si>
-  <si>
-    <t>Indica cada cuanto se revisa el indicador</t>
-  </si>
-  <si>
-    <t>Diario semanal por Sprint release y final</t>
-  </si>
-  <si>
-    <t>KRI-06</t>
+    <t>KRI-07</t>
+  </si>
+  <si>
+    <t>Registros con datos inconsistentes</t>
+  </si>
+  <si>
+    <t>≤2%</t>
+  </si>
+  <si>
+    <t>3%-5%</t>
+  </si>
+  <si>
+    <t>&gt;5%</t>
   </si>
   <si>
     <t>KPI-06</t>
   </si>
   <si>
-    <t>Cambios tardios del modelo de datos</t>
+    <t>Porcentaje</t>
+  </si>
+  <si>
+    <t>Unidad utilizada para medir cumplimiento cobertura calidad disponibilidad y error</t>
+  </si>
+  <si>
+    <t>Cobertura RF 90% y pruebas aprobadas 95%</t>
   </si>
   <si>
     <t>Cobertura RF verificados</t>
   </si>
   <si>
-    <t>Paulo</t>
-  </si>
-  <si>
-    <t>Persona o equipo encargado de revisar el indicador y coordinar acciones</t>
-  </si>
-  <si>
-    <t>Mauricio Paulo Alexander y Equipo</t>
-  </si>
-  <si>
-    <t>KRI-07</t>
+    <t>KRI-08</t>
+  </si>
+  <si>
+    <t>Consultas con tiempo excesivo</t>
+  </si>
+  <si>
+    <t>≤5%</t>
+  </si>
+  <si>
+    <t>6%-10%</t>
+  </si>
+  <si>
+    <t>&gt;10%</t>
+  </si>
+  <si>
+    <t>Conteo de eventos riesgos errores o elementos</t>
+  </si>
+  <si>
+    <t>Cantidad de bloqueos y defectos criticos</t>
+  </si>
+  <si>
+    <t>KRI-09</t>
   </si>
   <si>
     <t>KPI-07</t>
   </si>
   <si>
-    <t>Registros con datos inconsistentes</t>
+    <t>Migraciones fallidas</t>
   </si>
   <si>
     <t>Cobertura RNF verificados</t>
   </si>
   <si>
-    <t>≤2%</t>
-  </si>
-  <si>
     <t>≥85%</t>
   </si>
   <si>
-    <t>3%-5%</t>
-  </si>
-  <si>
-    <t>&gt;5%</t>
-  </si>
-  <si>
     <t>70%-84%</t>
   </si>
   <si>
     <t>&lt;70%</t>
   </si>
   <si>
-    <t>Porcentaje</t>
-  </si>
-  <si>
-    <t>Unidad utilizada para medir cumplimiento cobertura calidad disponibilidad y error</t>
-  </si>
-  <si>
-    <t>Cobertura RF 90% y pruebas aprobadas 95%</t>
-  </si>
-  <si>
-    <t>KRI-08</t>
-  </si>
-  <si>
-    <t>Consultas con tiempo excesivo</t>
+    <t>Release</t>
+  </si>
+  <si>
+    <t>Segundos</t>
+  </si>
+  <si>
+    <t>Unidad para medir tiempos de respuesta del sistema</t>
+  </si>
+  <si>
+    <t>Pantallas ≤3 segundos</t>
+  </si>
+  <si>
+    <t>KRI-10</t>
+  </si>
+  <si>
+    <t>Intentos de acceso entre companias</t>
   </si>
   <si>
     <t>KPI-08</t>
   </si>
   <si>
-    <t>≤5%</t>
-  </si>
-  <si>
     <t>Trazabilidad RF y RNF</t>
   </si>
   <si>
-    <t>6%-10%</t>
-  </si>
-  <si>
-    <t>&gt;10%</t>
-  </si>
-  <si>
-    <t>Conteo de eventos riesgos errores o elementos</t>
-  </si>
-  <si>
-    <t>Cantidad de bloqueos y defectos criticos</t>
-  </si>
-  <si>
-    <t>KRI-09</t>
-  </si>
-  <si>
-    <t>Migraciones fallidas</t>
+    <t>Diario</t>
+  </si>
+  <si>
+    <t>Horas</t>
+  </si>
+  <si>
+    <t>Unidad para tiempos de recuperacion y actividades cuando corresponda</t>
+  </si>
+  <si>
+    <t>Restauracion y correccion tecnica</t>
+  </si>
+  <si>
+    <t>KRI-11</t>
+  </si>
+  <si>
+    <t>Permisos incorrectos detectados</t>
   </si>
   <si>
     <t>KPI-09</t>
@@ -317,22 +383,19 @@
     <t>Pruebas planificadas ejecutadas</t>
   </si>
   <si>
-    <t>Release</t>
-  </si>
-  <si>
-    <t>Segundos</t>
-  </si>
-  <si>
-    <t>Unidad para medir tiempos de respuesta del sistema</t>
-  </si>
-  <si>
-    <t>Pantallas ≤3 segundos</t>
-  </si>
-  <si>
-    <t>KRI-10</t>
-  </si>
-  <si>
-    <t>Intentos de acceso entre companias</t>
+    <t>Dias</t>
+  </si>
+  <si>
+    <t>Unidad para medir duracion de bloqueos y ausencias</t>
+  </si>
+  <si>
+    <t>Bloqueo mayor a 2 dias</t>
+  </si>
+  <si>
+    <t>KRI-12</t>
+  </si>
+  <si>
+    <t>Accesos no autorizados</t>
   </si>
   <si>
     <t>KPI-10</t>
@@ -341,43 +404,79 @@
     <t>Pruebas ejecutadas aprobadas</t>
   </si>
   <si>
-    <t>Diario</t>
-  </si>
-  <si>
-    <t>Horas</t>
-  </si>
-  <si>
-    <t>Unidad para tiempos de recuperacion y actividades cuando corresponda</t>
-  </si>
-  <si>
-    <t>Restauracion y correccion tecnica</t>
-  </si>
-  <si>
-    <t>KRI-11</t>
-  </si>
-  <si>
-    <t>Permisos incorrectos detectados</t>
+    <t>Incidencias</t>
+  </si>
+  <si>
+    <t>Eventos que afectan el funcionamiento esperado</t>
+  </si>
+  <si>
+    <t>Inconsistencias de stock y problemas de coordinacion</t>
+  </si>
+  <si>
+    <t>KRI-13</t>
+  </si>
+  <si>
+    <t>Exposicion de credenciales</t>
+  </si>
+  <si>
+    <t>Resultado</t>
+  </si>
+  <si>
+    <t>Estado cualitativo utilizado cuando no corresponde un porcentaje</t>
+  </si>
+  <si>
+    <t>Aprobada Pendiente y Fallida</t>
+  </si>
+  <si>
+    <t>KRI-14</t>
+  </si>
+  <si>
+    <t>Historias que exceden capacidad del Sprint</t>
+  </si>
+  <si>
+    <t>Uptime</t>
+  </si>
+  <si>
+    <t>Porcentaje de tiempo disponible de un entorno o servicio</t>
+  </si>
+  <si>
+    <t>Disponibilidad entorno de desarrollo ≥95%</t>
   </si>
   <si>
     <t>KPI-11</t>
   </si>
   <si>
+    <t>KRI-15</t>
+  </si>
+  <si>
     <t>Defectos corregidos dentro del Sprint</t>
   </si>
   <si>
-    <t>Dias</t>
-  </si>
-  <si>
-    <t>Unidad para medir duracion de bloqueos y ausencias</t>
-  </si>
-  <si>
-    <t>Bloqueo mayor a 2 dias</t>
-  </si>
-  <si>
-    <t>KRI-12</t>
-  </si>
-  <si>
-    <t>Accesos no autorizados</t>
+    <t>Desviacion de estimacion de historias</t>
+  </si>
+  <si>
+    <t>≤20%</t>
+  </si>
+  <si>
+    <t>21%-35%</t>
+  </si>
+  <si>
+    <t>&gt;35%</t>
+  </si>
+  <si>
+    <t>Trazabilidad</t>
+  </si>
+  <si>
+    <t>Capacidad de relacionar requerimiento historia cambio prueba y evidencia</t>
+  </si>
+  <si>
+    <t>RF y RNF vinculados con prueba y resultado</t>
+  </si>
+  <si>
+    <t>KRI-16</t>
+  </si>
+  <si>
+    <t>Bloqueos activos por mas de 2 dias</t>
   </si>
   <si>
     <t>KPI-12</t>
@@ -386,19 +485,19 @@
     <t>Pruebas de regresion aprobadas</t>
   </si>
   <si>
-    <t>Incidencias</t>
-  </si>
-  <si>
-    <t>Eventos que afectan el funcionamiento esperado</t>
-  </si>
-  <si>
-    <t>Inconsistencias de stock y problemas de coordinacion</t>
-  </si>
-  <si>
-    <t>KRI-13</t>
-  </si>
-  <si>
-    <t>Exposicion de credenciales</t>
+    <t>Cobertura</t>
+  </si>
+  <si>
+    <t>Proporcion del alcance que cuenta con verificacion o prueba</t>
+  </si>
+  <si>
+    <t>Requisitos verificados sobre requisitos aplicables</t>
+  </si>
+  <si>
+    <t>KRI-17</t>
+  </si>
+  <si>
+    <t>Historias esenciales sin prioridad</t>
   </si>
   <si>
     <t>KPI-13</t>
@@ -410,64 +509,58 @@
     <t>% uptime</t>
   </si>
   <si>
+    <t>KRI-18</t>
+  </si>
+  <si>
+    <t>Trabajo pendiente frente a fecha final</t>
+  </si>
+  <si>
     <t>90%-94%</t>
   </si>
   <si>
-    <t>Resultado</t>
-  </si>
-  <si>
-    <t>Estado cualitativo utilizado cuando no corresponde un porcentaje</t>
-  </si>
-  <si>
-    <t>Aprobada Pendiente y Fallida</t>
-  </si>
-  <si>
-    <t>KRI-14</t>
-  </si>
-  <si>
-    <t>Historias que exceden capacidad del Sprint</t>
+    <t>≤10%</t>
+  </si>
+  <si>
+    <t>11%-20%</t>
+  </si>
+  <si>
+    <t>&gt;20%</t>
+  </si>
+  <si>
+    <t>KRI-19</t>
   </si>
   <si>
     <t>KPI-14</t>
   </si>
   <si>
+    <t>Ausencia de integrante en dias criticos</t>
+  </si>
+  <si>
     <t>Tiempo de respuesta de pantallas</t>
   </si>
   <si>
     <t>≤3</t>
   </si>
   <si>
-    <t>Uptime</t>
-  </si>
-  <si>
     <t>4-5</t>
   </si>
   <si>
-    <t>Porcentaje de tiempo disponible de un entorno o servicio</t>
-  </si>
-  <si>
-    <t>Disponibilidad entorno de desarrollo ≥95%</t>
-  </si>
-  <si>
     <t>&gt;5</t>
   </si>
   <si>
-    <t>KRI-15</t>
-  </si>
-  <si>
-    <t>Desviacion de estimacion de historias</t>
-  </si>
-  <si>
-    <t>≤20%</t>
-  </si>
-  <si>
-    <t>21%-35%</t>
+    <t>KRI-20</t>
+  </si>
+  <si>
+    <t>Dependencias de conocimiento en una persona</t>
+  </si>
+  <si>
+    <t>≤1</t>
   </si>
   <si>
     <t>KPI-15</t>
   </si>
   <si>
-    <t>&gt;35%</t>
+    <t>2</t>
   </si>
   <si>
     <t>Tiempo de carga de reportes</t>
@@ -476,43 +569,25 @@
     <t>≤5</t>
   </si>
   <si>
-    <t>Trazabilidad</t>
-  </si>
-  <si>
-    <t>Capacidad de relacionar requerimiento historia cambio prueba y evidencia</t>
-  </si>
-  <si>
-    <t>RF y RNF vinculados con prueba y resultado</t>
-  </si>
-  <si>
     <t>6-10</t>
   </si>
   <si>
     <t>&gt;10</t>
   </si>
   <si>
-    <t>KRI-16</t>
-  </si>
-  <si>
-    <t>Bloqueos activos por mas de 2 dias</t>
-  </si>
-  <si>
     <t>KPI-16</t>
   </si>
   <si>
     <t>Operaciones de inventario validas</t>
   </si>
   <si>
-    <t>Cobertura</t>
+    <t>KRI-21</t>
   </si>
   <si>
     <t>≥99%</t>
   </si>
   <si>
-    <t>Proporcion del alcance que cuenta con verificacion o prueba</t>
-  </si>
-  <si>
-    <t>Requisitos verificados sobre requisitos aplicables</t>
+    <t>Tareas criticas concentradas en una persona</t>
   </si>
   <si>
     <t>95%-98%</t>
@@ -521,49 +596,46 @@
     <t>&lt;95%</t>
   </si>
   <si>
-    <t>KRI-17</t>
-  </si>
-  <si>
-    <t>Historias esenciales sin prioridad</t>
-  </si>
-  <si>
     <t>KPI-17</t>
   </si>
   <si>
     <t>Exactitud de existencias</t>
   </si>
   <si>
-    <t>KRI-18</t>
-  </si>
-  <si>
-    <t>Trabajo pendiente frente a fecha final</t>
-  </si>
-  <si>
-    <t>≤10%</t>
-  </si>
-  <si>
-    <t>11%-20%</t>
+    <t>KRI-22</t>
+  </si>
+  <si>
+    <t>Problemas de coordinacion</t>
+  </si>
+  <si>
+    <t>2-3</t>
+  </si>
+  <si>
+    <t>≥4</t>
   </si>
   <si>
     <t>KPI-18</t>
   </si>
   <si>
+    <t>KRI-23</t>
+  </si>
+  <si>
+    <t>Inconsistencias de stock</t>
+  </si>
+  <si>
     <t>Articulos seriados sin duplicados</t>
   </si>
   <si>
-    <t>&gt;20%</t>
-  </si>
-  <si>
     <t>99%</t>
   </si>
   <si>
     <t>&lt;99%</t>
   </si>
   <si>
-    <t>KRI-19</t>
-  </si>
-  <si>
-    <t>Ausencia de integrante en dias criticos</t>
+    <t>KRI-24</t>
+  </si>
+  <si>
+    <t>Numeros de serie duplicados</t>
   </si>
   <si>
     <t>KPI-19</t>
@@ -575,10 +647,10 @@
     <t>95%-99%</t>
   </si>
   <si>
-    <t>KRI-20</t>
-  </si>
-  <si>
-    <t>Dependencias de conocimiento en una persona</t>
+    <t>KRI-25</t>
+  </si>
+  <si>
+    <t>Prestamos sin cierre correcto</t>
   </si>
   <si>
     <t>KPI-20</t>
@@ -587,16 +659,10 @@
     <t>Check in completados</t>
   </si>
   <si>
-    <t>≤1</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>KRI-21</t>
-  </si>
-  <si>
-    <t>Tareas criticas concentradas en una persona</t>
+    <t>KRI-26</t>
+  </si>
+  <si>
+    <t>Registros de unidad inconsistentes</t>
   </si>
   <si>
     <t>KPI-21</t>
@@ -605,28 +671,28 @@
     <t>Lecturas de unidad validas</t>
   </si>
   <si>
-    <t>KRI-22</t>
-  </si>
-  <si>
-    <t>Problemas de coordinacion</t>
+    <t>KRI-27</t>
+  </si>
+  <si>
+    <t>Alertas de mantenimiento incorrectas</t>
+  </si>
+  <si>
+    <t>KRI-28</t>
+  </si>
+  <si>
+    <t>Defectos criticos abiertos</t>
   </si>
   <si>
     <t>KPI-22</t>
   </si>
   <si>
-    <t>2-3</t>
-  </si>
-  <si>
     <t>Mantenimientos registrados con historial</t>
   </si>
   <si>
-    <t>≥4</t>
-  </si>
-  <si>
-    <t>KRI-23</t>
-  </si>
-  <si>
-    <t>Inconsistencias de stock</t>
+    <t>KRI-29</t>
+  </si>
+  <si>
+    <t>Pruebas no ejecutadas</t>
   </si>
   <si>
     <t>KPI-23</t>
@@ -635,10 +701,10 @@
     <t>Alertas de mantenimiento correctas</t>
   </si>
   <si>
-    <t>KRI-24</t>
-  </si>
-  <si>
-    <t>Numeros de serie duplicados</t>
+    <t>KRI-30</t>
+  </si>
+  <si>
+    <t>Dependencias externas sin resolver</t>
   </si>
   <si>
     <t>KPI-24</t>
@@ -647,27 +713,30 @@
     <t>Reportes generados sin error</t>
   </si>
   <si>
-    <t>KRI-25</t>
-  </si>
-  <si>
     <t>≥98%</t>
   </si>
   <si>
-    <t>Prestamos sin cierre correcto</t>
-  </si>
-  <si>
     <t>95%-97%</t>
   </si>
   <si>
-    <t>KRI-26</t>
+    <t>Nivel Risk Register</t>
+  </si>
+  <si>
+    <t>Responsable Risk Register</t>
+  </si>
+  <si>
+    <t>HIGHEST</t>
+  </si>
+  <si>
+    <t>HIGH</t>
+  </si>
+  <si>
+    <t>MEDIUM</t>
   </si>
   <si>
     <t>KPI-25</t>
   </si>
   <si>
-    <t>Registros de unidad inconsistentes</t>
-  </si>
-  <si>
     <t>Exportaciones Excel correctas</t>
   </si>
   <si>
@@ -711,45 +780,6 @@
   </si>
   <si>
     <t>Final</t>
-  </si>
-  <si>
-    <t>KRI-27</t>
-  </si>
-  <si>
-    <t>Alertas de mantenimiento incorrectas</t>
-  </si>
-  <si>
-    <t>KRI-28</t>
-  </si>
-  <si>
-    <t>Defectos criticos abiertos</t>
-  </si>
-  <si>
-    <t>KRI-29</t>
-  </si>
-  <si>
-    <t>Pruebas no ejecutadas</t>
-  </si>
-  <si>
-    <t>KRI-30</t>
-  </si>
-  <si>
-    <t>Dependencias externas sin resolver</t>
-  </si>
-  <si>
-    <t>Nivel Risk Register</t>
-  </si>
-  <si>
-    <t>Responsable Risk Register</t>
-  </si>
-  <si>
-    <t>HIGHEST</t>
-  </si>
-  <si>
-    <t>HIGH</t>
-  </si>
-  <si>
-    <t>MEDIUM</t>
   </si>
 </sst>
 </file>
@@ -880,6 +910,9 @@
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
@@ -887,9 +920,6 @@
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -952,13 +982,13 @@
     </dxf>
   </dxfs>
   <tableStyles count="2">
-    <tableStyle count="4" pivot="0" name="KPI-style">
+    <tableStyle count="4" pivot="0" name="KRI-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
       <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
     </tableStyle>
-    <tableStyle count="4" pivot="0" name="KRI-style">
+    <tableStyle count="4" pivot="0" name="KPI-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
@@ -1051,11 +1081,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1548056771"/>
-        <c:axId val="1276811992"/>
+        <c:axId val="1615493325"/>
+        <c:axId val="1748883353"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1548056771"/>
+        <c:axId val="1615493325"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1111,10 +1141,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1276811992"/>
+        <c:crossAx val="1748883353"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1276811992"/>
+        <c:axId val="1748883353"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1191,7 +1221,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1548056771"/>
+        <c:crossAx val="1615493325"/>
       </c:valAx>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
@@ -1282,11 +1312,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="170778295"/>
-        <c:axId val="312904399"/>
+        <c:axId val="1608045238"/>
+        <c:axId val="1318015876"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="170778295"/>
+        <c:axId val="1608045238"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1342,10 +1372,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="312904399"/>
+        <c:crossAx val="1318015876"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="312904399"/>
+        <c:axId val="1318015876"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1422,7 +1452,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="170778295"/>
+        <c:crossAx val="1608045238"/>
       </c:valAx>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
@@ -1513,11 +1543,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1936840220"/>
-        <c:axId val="1920912608"/>
+        <c:axId val="2005500358"/>
+        <c:axId val="1335641461"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1936840220"/>
+        <c:axId val="2005500358"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1573,10 +1603,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1920912608"/>
+        <c:crossAx val="1335641461"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1920912608"/>
+        <c:axId val="1335641461"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1653,7 +1683,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1936840220"/>
+        <c:crossAx val="2005500358"/>
       </c:valAx>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
@@ -1744,11 +1774,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="454410597"/>
-        <c:axId val="1833067160"/>
+        <c:axId val="1703207755"/>
+        <c:axId val="1220756472"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="454410597"/>
+        <c:axId val="1703207755"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1804,10 +1834,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1833067160"/>
+        <c:crossAx val="1220756472"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1833067160"/>
+        <c:axId val="1220756472"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1884,7 +1914,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="454410597"/>
+        <c:crossAx val="1703207755"/>
       </c:valAx>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
@@ -1904,7 +1934,7 @@
     <xdr:ext cx="5715000" cy="3048000"/>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 2" title="KPI por frecuencia"/>
+        <xdr:cNvPr id="1" name="Chart 1" title="KPI por frecuencia"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -1929,7 +1959,7 @@
     <xdr:ext cx="5715000" cy="3048000"/>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Chart 3" title="KPI por responsable"/>
+        <xdr:cNvPr id="4" name="Chart 4" title="KPI por responsable"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -1959,7 +1989,7 @@
     <xdr:ext cx="5715000" cy="3048000"/>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="1" name="Chart 1" title="Riesgos actuales por nivel"/>
+        <xdr:cNvPr id="2" name="Chart 2" title="Riesgos actuales por nivel"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -1984,7 +2014,7 @@
     <xdr:ext cx="5715000" cy="3048000"/>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 4" title="Riesgos actuales por responsable"/>
+        <xdr:cNvPr id="3" name="Chart 3" title="Riesgos actuales por responsable"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -2258,16 +2288,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>5</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>6</v>
@@ -2290,31 +2320,31 @@
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E2" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="H2" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G2" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>25</v>
-      </c>
       <c r="J2" s="8" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K2" s="8" t="s">
         <v>26</v>
@@ -2325,891 +2355,891 @@
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E3" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="K3" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="J3" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="K3" s="8" t="s">
-        <v>37</v>
-      </c>
       <c r="L3" s="8" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="K4" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="6" t="s">
+      <c r="L4" s="8" t="s">
         <v>43</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="J4" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="K4" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="L4" s="8" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="G5" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="H5" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="K5" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="5" t="s">
+      <c r="L5" s="8" t="s">
         <v>53</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="K5" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="L5" s="8" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="J6" s="8" t="s">
         <v>7</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="L6" s="8" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="3" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E7" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="H7" s="7" t="s">
         <v>23</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>25</v>
       </c>
       <c r="J7" s="8" t="s">
         <v>8</v>
       </c>
       <c r="K7" s="8" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="L7" s="8" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D8" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="K8" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="E8" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="J8" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="K8" s="8" t="s">
-        <v>86</v>
-      </c>
       <c r="L8" s="8" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J9" s="8" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K9" s="8" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="L9" s="8" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="K10" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="L10" s="8" t="s">
         <v>100</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="K10" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="L10" s="8" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="K11" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="L11" s="8" t="s">
         <v>108</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="K11" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="L11" s="8" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="K12" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="L12" s="8" t="s">
         <v>115</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="H12" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="J12" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="K12" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="L12" s="8" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="K13" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="L13" s="8" t="s">
         <v>122</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="J13" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="K13" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="L13" s="8" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="3" t="s">
-        <v>129</v>
+        <v>152</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>130</v>
+        <v>153</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>131</v>
+        <v>154</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>132</v>
+        <v>157</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="J14" s="8" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="K14" s="8" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="L14" s="8" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="3" t="s">
-        <v>138</v>
+        <v>162</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>139</v>
+        <v>164</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>140</v>
+        <v>165</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>142</v>
+        <v>166</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="J15" s="8" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="K15" s="8" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="L15" s="8" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="A16" s="3" t="s">
-        <v>150</v>
+        <v>171</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>153</v>
+        <v>174</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>157</v>
+        <v>175</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>158</v>
+        <v>176</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>154</v>
+        <v>140</v>
       </c>
       <c r="K16" s="8" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="L16" s="8" t="s">
-        <v>156</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17" ht="22.5" customHeight="1">
       <c r="A17" s="3" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>162</v>
+        <v>178</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>168</v>
+        <v>183</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="J17" s="8" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
       <c r="K17" s="8" t="s">
-        <v>165</v>
+        <v>148</v>
       </c>
       <c r="L17" s="8" t="s">
-        <v>166</v>
+        <v>149</v>
       </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
       <c r="A18" s="3" t="s">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>168</v>
+        <v>183</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19" ht="22.5" customHeight="1">
       <c r="A19" s="3" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>178</v>
+        <v>193</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>180</v>
+        <v>194</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>181</v>
+        <v>195</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" ht="22.5" customHeight="1">
       <c r="A20" s="3" t="s">
-        <v>184</v>
+        <v>198</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>185</v>
+        <v>199</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>186</v>
+        <v>200</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>168</v>
+        <v>183</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" ht="22.5" customHeight="1">
       <c r="A21" s="3" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="22" ht="22.5" customHeight="1">
       <c r="A22" s="3" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>168</v>
+        <v>183</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="23" ht="22.5" customHeight="1">
       <c r="A23" s="3" t="s">
-        <v>199</v>
+        <v>213</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>186</v>
+        <v>200</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>168</v>
+        <v>183</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24" ht="22.5" customHeight="1">
       <c r="A24" s="3" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="25" ht="22.5" customHeight="1">
       <c r="A25" s="3" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>168</v>
+        <v>183</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="26" ht="22.5" customHeight="1">
       <c r="A26" s="3" t="s">
-        <v>216</v>
+        <v>230</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>168</v>
+        <v>183</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="27" ht="22.5" customHeight="1">
       <c r="A27" s="3" t="s">
-        <v>219</v>
+        <v>232</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>220</v>
+        <v>233</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="28" ht="22.5" customHeight="1">
       <c r="A28" s="3" t="s">
-        <v>221</v>
+        <v>234</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="H28" s="7" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="29" ht="22.5" customHeight="1">
       <c r="A29" s="3" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="30" ht="22.5" customHeight="1">
       <c r="A30" s="3" t="s">
-        <v>228</v>
+        <v>241</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>229</v>
+        <v>242</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E30" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G30" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F30" s="5" t="s">
+      <c r="H30" s="7" t="s">
         <v>23</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H30" s="7" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="31" ht="22.5" customHeight="1">
       <c r="A31" s="3" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>232</v>
+        <v>245</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="32">
@@ -3221,7 +3251,7 @@
       <c r="G32" s="9"/>
     </row>
     <row r="33">
-      <c r="A33" s="10"/>
+      <c r="A33" s="11"/>
     </row>
     <row r="34">
       <c r="A34" s="9"/>
@@ -3232,35 +3262,35 @@
       <c r="G34" s="9"/>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="s">
+      <c r="A35" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="B35" s="11" t="s">
-        <v>16</v>
+      <c r="B35" s="12" t="s">
+        <v>14</v>
       </c>
       <c r="C35" s="9"/>
-      <c r="D35" s="11" t="s">
+      <c r="D35" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="E35" s="11" t="s">
-        <v>16</v>
+      <c r="E35" s="12" t="s">
+        <v>14</v>
       </c>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
     </row>
     <row r="36">
-      <c r="A36" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="B36" s="12">
+      <c r="A36" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="B36" s="13">
         <f t="shared" ref="B36:B40" si="1">COUNTIF($G$2:$G$31,A36)</f>
         <v>0</v>
       </c>
       <c r="C36" s="9"/>
-      <c r="D36" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="E36" s="12">
+      <c r="D36" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="E36" s="13">
         <f t="shared" ref="E36:E39" si="2">COUNTIF($H$2:$H$31,D36)</f>
         <v>10</v>
       </c>
@@ -3268,18 +3298,18 @@
       <c r="G36" s="9"/>
     </row>
     <row r="37">
-      <c r="A37" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="B37" s="12">
+      <c r="A37" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B37" s="13">
         <f t="shared" si="1"/>
         <v>14</v>
       </c>
       <c r="C37" s="9"/>
-      <c r="D37" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="E37" s="12">
+      <c r="D37" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="E37" s="13">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
@@ -3287,18 +3317,18 @@
       <c r="G37" s="9"/>
     </row>
     <row r="38">
-      <c r="A38" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="B38" s="12">
+      <c r="A38" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="B38" s="13">
         <f t="shared" si="1"/>
         <v>14</v>
       </c>
       <c r="C38" s="9"/>
-      <c r="D38" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="E38" s="12">
+      <c r="D38" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E38" s="13">
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
@@ -3306,18 +3336,18 @@
       <c r="G38" s="9"/>
     </row>
     <row r="39">
-      <c r="A39" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="B39" s="12">
+      <c r="A39" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="B39" s="13">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="C39" s="9"/>
-      <c r="D39" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="E39" s="12">
+      <c r="D39" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="E39" s="13">
         <f t="shared" si="2"/>
         <v>6</v>
       </c>
@@ -3325,10 +3355,10 @@
       <c r="G39" s="9"/>
     </row>
     <row r="40">
-      <c r="A40" s="12" t="s">
-        <v>232</v>
-      </c>
-      <c r="B40" s="12">
+      <c r="A40" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="B40" s="13">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
@@ -11017,9 +11047,10 @@
   <dataValidations>
     <dataValidation allowBlank="1" showDropDown="1" sqref="A2:H31"/>
   </dataValidations>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
@@ -11053,13 +11084,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>5</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>6</v>
@@ -11085,28 +11116,28 @@
         <v>12</v>
       </c>
       <c r="B2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="E2" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="6" t="s">
-        <v>20</v>
-      </c>
       <c r="F2" s="5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K2" s="8" t="s">
         <v>26</v>
@@ -11120,888 +11151,888 @@
         <v>28</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>33</v>
-      </c>
       <c r="F3" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="L3" s="8" t="s">
         <v>35</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="J3" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="K3" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="L3" s="8" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="J4" s="8" t="s">
-        <v>46</v>
-      </c>
       <c r="K4" s="8" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J5" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>56</v>
-      </c>
       <c r="K5" s="8" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="L5" s="8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="6" t="s">
-        <v>20</v>
-      </c>
       <c r="F6" s="5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="J6" s="8" t="s">
         <v>7</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="L6" s="8" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H7" s="7" t="s">
         <v>68</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>72</v>
       </c>
       <c r="J7" s="8" t="s">
         <v>8</v>
       </c>
       <c r="K7" s="8" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="L7" s="8" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="E8" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="5" t="s">
+      <c r="G8" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="J8" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="K8" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="L8" s="8" t="s">
         <v>81</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="J8" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="K8" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="L8" s="8" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="K9" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="L9" s="8" t="s">
         <v>89</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="K9" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="L9" s="8" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G10" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="H10" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="J10" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>102</v>
-      </c>
       <c r="K10" s="8" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="L10" s="8" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="H11" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="J11" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>110</v>
-      </c>
       <c r="K11" s="8" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="L11" s="8" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="J12" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="K12" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="H12" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="J12" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="K12" s="8" t="s">
-        <v>118</v>
-      </c>
       <c r="L12" s="8" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="J13" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="K13" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="C13" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="J13" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="K13" s="8" t="s">
-        <v>125</v>
-      </c>
       <c r="L13" s="8" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="J14" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="K14" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="L14" s="8" t="s">
         <v>127</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H14" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="J14" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="K14" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="L14" s="8" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="3" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="C15" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D15" s="6" t="s">
-        <v>18</v>
-      </c>
       <c r="E15" s="6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J15" s="8" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="K15" s="8" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="L15" s="8" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="A16" s="3" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>154</v>
+        <v>140</v>
       </c>
       <c r="K16" s="8" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="L16" s="8" t="s">
-        <v>156</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17" ht="22.5" customHeight="1">
       <c r="A17" s="3" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="C17" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D17" s="6" t="s">
-        <v>18</v>
-      </c>
       <c r="E17" s="6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J17" s="8" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
       <c r="K17" s="8" t="s">
-        <v>165</v>
+        <v>148</v>
       </c>
       <c r="L17" s="8" t="s">
-        <v>166</v>
+        <v>149</v>
       </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
       <c r="A18" s="3" t="s">
-        <v>169</v>
+        <v>150</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>170</v>
+        <v>151</v>
       </c>
       <c r="C18" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="6" t="s">
-        <v>18</v>
-      </c>
       <c r="E18" s="6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" ht="22.5" customHeight="1">
       <c r="A19" s="3" t="s">
-        <v>173</v>
+        <v>155</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>174</v>
+        <v>156</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>175</v>
+        <v>158</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>176</v>
+        <v>159</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>179</v>
+        <v>160</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20" ht="22.5" customHeight="1">
       <c r="A20" s="3" t="s">
-        <v>182</v>
+        <v>161</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" ht="22.5" customHeight="1">
       <c r="A21" s="3" t="s">
-        <v>187</v>
+        <v>168</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>188</v>
+        <v>169</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>191</v>
+        <v>170</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="22" ht="22.5" customHeight="1">
       <c r="A22" s="3" t="s">
-        <v>193</v>
+        <v>179</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>140</v>
+        <v>165</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>142</v>
+        <v>166</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="23" ht="22.5" customHeight="1">
       <c r="A23" s="3" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>191</v>
+        <v>170</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>202</v>
+        <v>189</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="24" ht="22.5" customHeight="1">
       <c r="A24" s="3" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="25" ht="22.5" customHeight="1">
       <c r="A25" s="3" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="C25" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D25" s="6" t="s">
-        <v>18</v>
-      </c>
       <c r="E25" s="6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="26" ht="22.5" customHeight="1">
       <c r="A26" s="3" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="C26" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D26" s="6" t="s">
-        <v>18</v>
-      </c>
       <c r="E26" s="6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="27" ht="22.5" customHeight="1">
       <c r="A27" s="3" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
       <c r="C27" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D27" s="6" t="s">
-        <v>18</v>
-      </c>
       <c r="E27" s="6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="28" ht="22.5" customHeight="1">
       <c r="A28" s="3" t="s">
-        <v>233</v>
+        <v>209</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>234</v>
+        <v>210</v>
       </c>
       <c r="C28" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D28" s="6" t="s">
+      <c r="E28" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E28" s="6" t="s">
-        <v>20</v>
-      </c>
       <c r="F28" s="5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H28" s="7" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="29" ht="22.5" customHeight="1">
       <c r="A29" s="3" t="s">
-        <v>235</v>
+        <v>211</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>236</v>
+        <v>212</v>
       </c>
       <c r="C29" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D29" s="6" t="s">
-        <v>18</v>
-      </c>
       <c r="E29" s="6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="30" ht="22.5" customHeight="1">
       <c r="A30" s="3" t="s">
-        <v>237</v>
+        <v>215</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>238</v>
+        <v>216</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>175</v>
+        <v>158</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>176</v>
+        <v>159</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>179</v>
+        <v>160</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="31" ht="22.5" customHeight="1">
       <c r="A31" s="3" t="s">
-        <v>239</v>
+        <v>219</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="C31" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D31" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="E31" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E31" s="6" t="s">
-        <v>20</v>
-      </c>
       <c r="F31" s="5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="32">
@@ -12013,10 +12044,10 @@
       <c r="G32" s="9"/>
     </row>
     <row r="33">
-      <c r="A33" s="13"/>
+      <c r="A33" s="10"/>
     </row>
     <row r="34">
-      <c r="A34" s="10"/>
+      <c r="A34" s="11"/>
     </row>
     <row r="35">
       <c r="A35" s="9"/>
@@ -12027,68 +12058,68 @@
       <c r="G35" s="9"/>
     </row>
     <row r="36">
-      <c r="A36" s="11" t="s">
-        <v>241</v>
-      </c>
-      <c r="B36" s="11" t="s">
-        <v>16</v>
+      <c r="A36" s="12" t="s">
+        <v>225</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>14</v>
       </c>
       <c r="C36" s="9"/>
-      <c r="D36" s="11" t="s">
-        <v>242</v>
-      </c>
-      <c r="E36" s="11" t="s">
-        <v>16</v>
+      <c r="D36" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="E36" s="12" t="s">
+        <v>14</v>
       </c>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
     </row>
     <row r="37">
-      <c r="A37" s="12" t="s">
-        <v>243</v>
-      </c>
-      <c r="B37" s="12">
+      <c r="A37" s="13" t="s">
+        <v>227</v>
+      </c>
+      <c r="B37" s="13">
         <v>1.0</v>
       </c>
       <c r="C37" s="9"/>
-      <c r="D37" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="E37" s="12">
+      <c r="D37" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="E37" s="13">
         <v>17.0</v>
       </c>
       <c r="F37" s="9"/>
       <c r="G37" s="9"/>
     </row>
     <row r="38">
-      <c r="A38" s="12" t="s">
-        <v>244</v>
-      </c>
-      <c r="B38" s="12">
+      <c r="A38" s="13" t="s">
+        <v>228</v>
+      </c>
+      <c r="B38" s="13">
         <v>32.0</v>
       </c>
       <c r="C38" s="9"/>
-      <c r="D38" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="E38" s="12">
+      <c r="D38" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="E38" s="13">
         <v>15.0</v>
       </c>
       <c r="F38" s="9"/>
       <c r="G38" s="9"/>
     </row>
     <row r="39">
-      <c r="A39" s="12" t="s">
-        <v>245</v>
-      </c>
-      <c r="B39" s="12">
+      <c r="A39" s="13" t="s">
+        <v>229</v>
+      </c>
+      <c r="B39" s="13">
         <v>7.0</v>
       </c>
       <c r="C39" s="9"/>
-      <c r="D39" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="E39" s="12">
+      <c r="D39" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E39" s="13">
         <v>8.0</v>
       </c>
       <c r="F39" s="9"/>
@@ -19786,9 +19817,10 @@
   <dataValidations>
     <dataValidation allowBlank="1" showDropDown="1" sqref="A2:H31"/>
   </dataValidations>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>